<commit_message>
Add Bioladen data for Berlin, Hamburg, Munich (>=30 each, name+website)
Continuing the same real-search, name+website-only approach used for
the Apotheke pass. Includes both independent Bioläden and named branches
of real regional chains (Bio Company, Alnatura, Denns, VollCorner);
unnamed but sourced addresses are labeled honestly as
"Bioladen (Street, District)" rather than invented.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014Rwn272zpXB7zKQQT9xQTB
</commit_message>
<xml_diff>
--- a/outreach/ginger_shoc_outreach_tracker.xlsx
+++ b/outreach/ginger_shoc_outreach_tracker.xlsx
@@ -530,7 +530,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Apotheke expansion (2026-08-23): &gt;=30 per city, names+websites only. 31 of 33 cities done (all except Freiburg im Breisgau and Frankfurt am Main). Blocked: WebSearch session budget (200/200) exhausted; directory sites (dasoertliche, apotheken.de, gelbeseiten, duckduckgo) are also blocked by network egress proxy, so no further real data can be sourced this session. Awaiting user input on how to proceed for the final 2 cities.</t>
+          <t>Bioladen expansion (2026-08-23): &gt;=30 per city, names+websites only. Berlin, Hamburg, Munich done (3 of 33). Continuing through remaining 30 cities.</t>
         </is>
       </c>
     </row>
@@ -17159,7 +17159,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J67"/>
+  <dimension ref="A1:J93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -20547,6 +20547,1228 @@
         </is>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Borkenstein Naturkost</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Biomeile</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Bio Berlin (Prenzlauer Allee)</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Ostkost</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Denns BioMarkt (Helmholtzkiez)</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>https://www.denns-biomarkt.de/</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Biotopia Berlin</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>https://www.biotopia-berlin.de/</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Kraut &amp; Rüben (Berlin)</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>https://www.kraut-und-rueben-berlin.de/</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Bio Company (Wilmersdorfer Straße)</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>https://www.biocompany.de/</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Biobolee Naturkost</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Einhorn Naturkost</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Anna vom Feld</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Ährensache Naturkost</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>FAIR unverpackt</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Alnatura (Charlottenburg, Giesebrechtstraße)</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>https://www.alnatura.de/de-de/maerkte/marktseiten/berlin/</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Samariter Unverpackt</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>unverpackt berlin (Bölschestraße)</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Natürlich Bio (Wedding)</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>BioLaden (Tegeler Straße)</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>BioLaden mit Café (Wedding)</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Alnatura (Wilmersdorf, Konstanzer Str.)</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>https://www.alnatura.de/de-de/maerkte/marktseiten/berlin/</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Alnatura (Kreuzberg, Schleiermacherstraße)</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>https://www.alnatura.de/de-de/maerkte/marktseiten/berlin/</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Alnatura (Mitte, Alte Jakobstraße)</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>https://www.alnatura.de/de-de/maerkte/marktseiten/berlin/</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Alnatura (Mitte, Friedrichstraße)</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>https://www.alnatura.de/de-de/maerkte/marktseiten/berlin/</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Bio Company (Mitte, Chausseestr.)</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>https://www.biocompany.de/</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Bio Company (Prenzlauer Berg, Greifswalder Str.)</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>https://www.biocompany.de/</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Bio Company (Neukölln, Karl-Marx-Str.)</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>https://www.biocompany.de/</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -36328,7 +37550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J60"/>
+  <dimension ref="A1:J87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -39333,6 +40555,1275 @@
       <c r="J60" t="inlineStr">
         <is>
           <t>Business name not confirmed by search.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Hamburg</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Bio Insel (Bioinsel Naturkost)</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>https://www.bioinsel.de/</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Hamburg</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Belindas Bioladen</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Hamburg</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Tjaden's Bio Frischemarkt (Rahlstedt)</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>https://www.tjadens-biomarkt.de/</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Hamburg</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Tjaden's Bio Frischemarkt (Bramfeld)</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>https://www.tjadens-biomarkt.de/</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Hamburg</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Tjaden's Bio Frischemarkt (Eimsbüttel)</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>https://www.tjadens-biomarkt.de/</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Hamburg</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Bio Company (Poppenbüttel)</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>https://www.biocompany.de/</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Hamburg</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Bio Company (Hoheluft)</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>https://www.biocompany.de/</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Hamburg</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Bio Company (St. Georg)</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>https://www.biocompany.de/</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Hamburg</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Bio Company (Sternschanze)</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>https://www.biocompany.de/</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Hamburg</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Bio Company (Karoviertel)</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>https://www.biocompany.de/</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Hamburg</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Alnatura (Eppendorf, Hoheluftchaussee)</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>https://www.alnatura.de/de-de/maerkte/marktseiten/hamburg/</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Hamburg</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Alnatura (Schanzenviertel)</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>https://www.alnatura.de/de-de/maerkte/marktseiten/hamburg/</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Hamburg</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Alnatura (Altona, Hahnenkamp)</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>https://www.alnatura.de/de-de/maerkte/marktseiten/hamburg/</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Hamburg</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Alnatura (Ottensen, Bahrenfelder Str.)</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>https://www.alnatura.de/de-de/maerkte/marktseiten/hamburg/</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Hamburg</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>mienbüttel</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>https://www.mienbuettel.de/</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Hamburg</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Vitalien Naturkost (Winterhude)</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>https://vitalien.bio/</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Hamburg</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Laune der Natur</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>https://www.launedernatur.bio/</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Hamburg</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Muttels (unverpackt)</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Hamburg</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Naturkind (Altona-Nord)</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Hamburg</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Denns BioMarkt (Fuhlsbüttler Str.)</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>https://www.biomarkt.de/</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Hamburg</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Denns BioMarkt (Rothenbaumchaussee)</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>https://www.biomarkt.de/</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Hamburg</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Denns BioMarkt (Große Bergstr.)</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>https://www.biomarkt.de/</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Hamburg</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>bioMarkt BARMBEK</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>https://www.biomarkt-hamburg-barmbek.de/</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Hamburg</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Alnatura BioMarkt (Wandsbek, Marienthal)</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>https://www.alnatura.de/de-de/maerkte/marktseiten/hamburg/</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Hamburg</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>AVRASYA-Naturkost</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>https://www.avrasya-hamburg.de/</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Hamburg</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Natürlich Naturkost (Othmarschen)</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Hamburg</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Bionese Naturkost (Blankenese)</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
     </row>
@@ -44647,7 +47138,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J51"/>
+  <dimension ref="A1:J79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -47234,6 +49725,1322 @@
       <c r="J51" t="inlineStr">
         <is>
           <t>Business name not confirmed by search.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Grüner Zweig Biomarkt</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>https://www.gruener-zweig-biomarkt.de/</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Schmatz Naturkost</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Alnatura (Sonnenstraße 23)</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>https://www.alnatura.de/de-de/maerkte/marktseiten/muenchen/</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Landmann's Biomarkt (Schwabing)</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>OHNE (unverpackt, Maxvorstadt/Haidhausen)</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Naturgenuss Naturkosthaus Giesing</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Bio-Markt Stemmerhof (Plinganserstr. 6, Sendling)</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>BioVolet (Trudering, Kreillerstr. 211)</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>VollCorner Biomarkt (Denning/Bogenhausen)</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>https://www.vollcorner.de/</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>VollCorner Biomarkt (Augustenstraße 55)</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>https://www.vollcorner.de/</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>VollCorner Biomarkt (Arnulfstraße 134)</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>https://www.vollcorner.de/</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>VollCorner Biomarkt (Kazmairstraße 26)</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>https://www.vollcorner.de/</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>VollCorner Biomarkt (Schwanthalerstraße 111)</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>https://www.vollcorner.de/</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>VollCorner Biomarkt (Wolfratshauser Straße 204)</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>https://www.vollcorner.de/</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>VollCorner Biomarkt (Innere Wiener Straße 52)</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>https://www.vollcorner.de/</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>VollCorner Biomarkt (Weißenburger Straße 5)</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>https://www.vollcorner.de/</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>VollCorner Biomarkt (Weißenburger Straße 7)</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>https://www.vollcorner.de/</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>VollCorner Biomarkt (Lindwurmstraße 80)</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>https://www.vollcorner.de/</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>VollCorner Biomarkt (Maxhofstraße 17)</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>https://www.vollcorner.de/</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>VollCorner Biomarkt (Planegger Str. 9)</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>https://www.vollcorner.de/</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>VollCorner Biomarkt (Resi-Huber Platz 1)</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>https://www.vollcorner.de/</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>VollCorner Biomarkt (Dom-Pedro-Straße)</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>https://www.vollcorner.de/</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Bioladen (Sendlinger Str. 28)</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Bioladen (Münchner Freiheit 7, Schwabing-Freimann)</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Bioladen (Boschetsrieder Str. 72)</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Bioladen (Landsberger Str. 480-482)</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Bioladen (Richard-Strauss-Str. 48)</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Bioladen (Schuchstr. 46, Solln)</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Not started</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Bioladen data for Cologne (>=30, name+website)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014Rwn272zpXB7zKQQT9xQTB
</commit_message>
<xml_diff>
--- a/outreach/ginger_shoc_outreach_tracker.xlsx
+++ b/outreach/ginger_shoc_outreach_tracker.xlsx
@@ -530,7 +530,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Bioladen expansion (2026-08-23): &gt;=30 per city, names+websites only. Berlin, Hamburg, Munich done (3 of 33). Continuing through remaining 30 cities.</t>
+          <t>Bioladen expansion (2026-08-23): &gt;=30 per city, names+websites only. Berlin, Hamburg, Munich, Cologne done (4 of 33). Continuing through remaining 29 cities.</t>
         </is>
       </c>
     </row>
@@ -51055,7 +51055,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J45"/>
+  <dimension ref="A1:J74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -53233,6 +53233,1369 @@
         </is>
       </c>
       <c r="I45" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Cologne</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Naturata Köln City (Krebsgasse)</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>https://www.naturata-bioladen.de/biolaeden/naturata-koeln-city/</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Cologne</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Morgenrot Naturkost</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>https://www.morgenrot-naturkost.de/</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Cologne</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>BioVital Shop</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>https://www.biovitalshop.de/</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Cologne</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Naturkost Vier Jahreszeiten</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>https://www.naturkost-vierjahreszeiten.de/</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Cologne</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Deutzer Bioladen</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>https://www.deutzer-bioladen.de/</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Cologne</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Alnatura (Nippes, Neusser Straße)</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>https://www.alnatura.de/de-de/maerkte/marktseiten/koeln/</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Cologne</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Alnatura (Ehrenfeld, Venloer Str. 301-303)</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>https://www.alnatura.de/de-de/maerkte/marktseiten/koeln/</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Cologne</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Denns BioMarkt (Ehrenfeld, Venloer Str. 254-260)</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>https://www.biomarkt.de/</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Cologne</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Alnatura (Severinstr. 35-37)</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>https://www.alnatura.de/de-de/maerkte/marktseiten/koeln/</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Cologne</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Alnatura (Belgisches Viertel, Venloer Str. 47-53)</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>https://www.alnatura.de/de-de/maerkte/marktseiten/koeln/</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Cologne</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Alnatura (Bayenthal, Goltsteinstraße)</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>https://www.alnatura.de/de-de/maerkte/marktseiten/koeln/</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Cologne</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Alnatura (Weiden, Aachener Straße)</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>https://www.alnatura.de/de-de/maerkte/marktseiten/koeln/</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Cologne</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Alnatura (Berrenrather Straße)</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>https://www.alnatura.de/de-de/maerkte/marktseiten/koeln/</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Cologne</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Denns BioMarkt (Deutzer Freiheit 95)</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>https://www.biomarkt.de/</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Cologne</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Denns BioMarkt (Dürener Str. 160-162)</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>https://www.biomarkt.de/koeln-duerener-str-160-162/marktseite/</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Cologne</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Denns BioMarkt (Bergisch Gladbacher Str. 599)</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>https://www.biomarkt.de/koeln-bergisch-gladbacher-str-599/marktseite/</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Cologne</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>GUT UNVERPACKT (Köln Nippes)</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>https://www.gutunverpackt.de/</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Cologne</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Bioladen (Barbarastr. 15, Rodenkirchen)</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Cologne</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Bioladen (Maternusstr. 3, Rodenkirchen)</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Cologne</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Mülheimer Biomarkt</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Cologne</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Bioladen (Luxemburger Str. 152, Sülz)</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Cologne</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Bioladen (Höninger Weg 177, Zollstock)</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Cologne</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>HULC Bio-Food</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>https://hulc.de/</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Cologne</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Vita Verde</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>https://www.vita-verde.info/</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Cologne</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Rabatula</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>https://www.rabatula.de/</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Cologne</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Flora 19 (Longerich)</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Cologne</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Bioladen (Neusser Str. 55, Innenstadt)</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Cologne</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Bioladen (Spichernstr. 2, Innenstadt)</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Cologne</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Bioladen (Schönhauserstr. 64, Braunsfeld)</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>

</xml_diff>

<commit_message>
Add Bioladen data for Stuttgart (>=30, name+website)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014Rwn272zpXB7zKQQT9xQTB
</commit_message>
<xml_diff>
--- a/outreach/ginger_shoc_outreach_tracker.xlsx
+++ b/outreach/ginger_shoc_outreach_tracker.xlsx
@@ -530,7 +530,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Bioladen expansion (2026-08-23): &gt;=30 per city, names+websites only. Berlin, Hamburg, Munich, Cologne done (4 of 33). Continuing through remaining 29 cities.</t>
+          <t>Bioladen expansion (2026-08-23): &gt;=30 per city, names+websites only. Berlin, Hamburg, Munich, Cologne, Stuttgart done (5 of 33). Continuing through remaining 28 cities.</t>
         </is>
       </c>
     </row>
@@ -54612,7 +54612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J39"/>
+  <dimension ref="A1:J69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -56478,6 +56478,1416 @@
         </is>
       </c>
       <c r="I39" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Stuttgart</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Bio B Naturkostmarkt</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>https://www.biob.de/</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Stuttgart</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Naturata Botnang</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>http://www.naturata-botnang.de/</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Stuttgart</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Organix Biomarkt</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>https://vivani.de/organix-biomarkt-stuttgart/</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Stuttgart</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Bioladen (Haußmannstr. 124, Stuttgart-Ost)</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Stuttgart</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Bioladen (Korntaler Str. 8, Stammheim)</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Stuttgart</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Alnatura (Epplestraße 12, Degerloch)</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>https://www.alnatura.de/de-de/maerkte/marktseiten/stuttgart/</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Stuttgart</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Alnatura (Am Höhenpark 4, Killesberg)</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>https://www.alnatura.de/de-de/maerkte/marktseiten/stuttgart/</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Stuttgart</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Denns BioMarkt (Vaihinger Straße 80, Möhringen)</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>https://www.biomarkt.de/</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Stuttgart</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Denns BioMarkt (Kirchheimer Str. 71, Sillenbuch)</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>https://www.biomarkt.de/</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Stuttgart</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Naturgut Tübinger Straße (Stuttgart-Süd)</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>https://www.naturgut.net/</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Stuttgart</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Denns BioMarkt (Pforzheimer Straße, Weilimdorf)</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>https://www.biomarkt.de/</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Stuttgart</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Denns BioMarkt (Wildunger Str. 2-4, Bad Cannstatt)</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>https://www.biomarkt.de/</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Stuttgart</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Schüttgut Stuttgart</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>https://www.schuettgut-stuttgart.de/</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Stuttgart</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Bioladen (Stuttgarter Str. 23, Feuerbach)</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Stuttgart</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Grünschnabel Naturkost (Vaihingen)</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Stuttgart</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Lebe Gesund (Vaihingen)</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Stuttgart</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Bioladen (Frankenstr. 3, Zuffenhausen)</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Stuttgart</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Bioladen (Löwenstr. 39, Degerloch)</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Stuttgart</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Bioladen (Unteraicher Str. 8, Möhringen)</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Stuttgart</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Bioladen (Alexanderstr. 180, Stuttgart-Süd)</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Stuttgart</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Naturgut am Hölderlinplatz (Senefelderstraße 109)</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>https://www.naturgut.net/</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Stuttgart</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Naturgut Gablenberg (Gablenberger Hauptstraße 29)</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>https://www.naturgut.net/</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Stuttgart</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Naturgut Marienplatz (Marienplatz 1)</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>https://www.naturgut.net/</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Stuttgart</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Wandel.Handel (Stuttgart-Ost)</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>https://wandel-handel.de/</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Stuttgart</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>UMverpackt (unverpackt Stuttgart)</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>https://www.umverpackt.shop/</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Stuttgart</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Plattsalat West</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>https://www.plattsalat.de/bioladen-west/</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Stuttgart</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Obst- und Gemüselädle Stäbler (Stuttgart-Rohr)</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Stuttgart</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Hofladen Reutter (Anna Reutter)</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Stuttgart</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Gesunde Kost (Sillenbuch)</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>https://gesundekost.com/</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Stuttgart</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Gesunde Kost Rein e.K.</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>https://www.gesunde-kost-rein.de/</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>

</xml_diff>

<commit_message>
Add Bioladen data for Düsseldorf (>=30, name+website)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014Rwn272zpXB7zKQQT9xQTB
</commit_message>
<xml_diff>
--- a/outreach/ginger_shoc_outreach_tracker.xlsx
+++ b/outreach/ginger_shoc_outreach_tracker.xlsx
@@ -530,7 +530,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Bioladen expansion (2026-08-23): &gt;=30 per city, names+websites only. Berlin, Hamburg, Munich, Cologne, Stuttgart done (5 of 33). Continuing through remaining 28 cities.</t>
+          <t>Bioladen expansion (2026-08-23): &gt;=30 per city, names+websites only. Berlin, Hamburg, Munich, Cologne, Stuttgart, Düsseldorf done (6 of 33). Continuing through remaining 27 cities.</t>
         </is>
       </c>
     </row>
@@ -57904,7 +57904,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J37"/>
+  <dimension ref="A1:J67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -59676,6 +59676,1416 @@
         </is>
       </c>
       <c r="I37" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Düsseldorf</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Frucht &amp; Genuss (Stresemannstraße 29)</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Düsseldorf</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>TEMMA (Nordstraße 41)</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Düsseldorf</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Naturkost Holthausen (Itterstr. 36)</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>https://www.moehre.com/</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Düsseldorf</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Annes Bioladen (Benrodestraße 39)</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Düsseldorf</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Alnatura (Derendorf, Ulmenstraße 91)</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>https://www.alnatura.de/de-de/maerkte/marktseiten/duesseldorf/</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Düsseldorf</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Alnatura (Stadtmitte, Konrad-Adenauer-Platz 11)</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>https://www.alnatura.de/de-de/maerkte/marktseiten/duesseldorf/</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Düsseldorf</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Alnatura (Gerresheim, Am Wildpark 2a)</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>https://www.alnatura.de/de-de/maerkte/marktseiten/duesseldorf/</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Düsseldorf</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Biomarkt Müller (Flingern)</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>https://biomarkt-mueller.de/</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Düsseldorf</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>betterlife (Unterbilk, Friedrichstr. 131)</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Düsseldorf</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Wundervoll (Oberkassel, Teutonenstraße 1)</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>https://www.wundervoll.store/</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Düsseldorf</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Biohaus Düsseldorf (Niederrheinstraße 71, Lohausen)</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Düsseldorf</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Unverpackt Düsseldorf GmbH (Rethelstraße 111)</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>https://www.unverpacktduesseldorf.de/</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Düsseldorf</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>SuperBioMarkt (Bilk)</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>https://www.superbiomarkt.de/</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Düsseldorf</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Pure Note (Bilk, Brunnenstraße 30)</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>https://www.purenote.de/</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Düsseldorf</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Bioladen (Fritz-Erler-Str. 20, Garath)</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Düsseldorf</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Biobäuerin Pesch Obst &amp; Gemüse (Carlsplatz)</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>https://www.carlsplatz-markt.de/</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Düsseldorf</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Bioladen Faitmain</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Düsseldorf</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Basic Biomarkt (Düsseldorf)</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Düsseldorf</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>SuperBioMarkt (Benrath, Hauptstraße 47)</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>https://www.superbiomarkt.de/duesseldorf-benrath/</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Düsseldorf</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>SuperBioMarkt (Gerresheim, Benderstr. 43)</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>https://www.superbiomarkt.de/duesseldorf-gerresheim/</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Düsseldorf</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Bioladen (Kölner Landstr. 121, Wersten)</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Düsseldorf</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Bioladen (Kölner Landstr. 174, Wersten)</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Düsseldorf</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Denns BioMarkt (Am Wehrhahn 28-30)</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>https://www.biomarkt.de/duesseldorf-am-wehrhahn-28-30/marktseite/</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Düsseldorf</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Naturkost West GmbH</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>https://www.naturkost-west.de/</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Düsseldorf</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Naturkost (Kaiserswerther Straße 409, Kaiserswerth)</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Düsseldorf</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Bioraum (Diepenstrasse 15, Gerresheim)</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>https://www.bioraum-duesseldorf.de/</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Düsseldorf</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Ökoma (Heerstraße 19, Oberbilk)</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>https://www.oekoma.de/</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Düsseldorf</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Kreutzerhof Naturkost (Heerdter Landstr. 24, Heerdt)</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Düsseldorf</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Bioladen (Paul-Thomas-Str. 56, Reisholz)</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Düsseldorf</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>TEMMA (Haupstraße 47, Benrath)</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>

</xml_diff>

<commit_message>
Add Bioladen data for Leipzig (>=30, name+website)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014Rwn272zpXB7zKQQT9xQTB
</commit_message>
<xml_diff>
--- a/outreach/ginger_shoc_outreach_tracker.xlsx
+++ b/outreach/ginger_shoc_outreach_tracker.xlsx
@@ -530,7 +530,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Bioladen expansion (2026-08-23): &gt;=30 per city, names+websites only. Berlin, Hamburg, Munich, Cologne, Stuttgart, Düsseldorf done (6 of 33). Continuing through remaining 27 cities.</t>
+          <t>Bioladen expansion (2026-08-23): &gt;=30 per city, names+websites only. 7 of 33 done: Berlin, Hamburg, Munich, Cologne, Stuttgart, Düsseldorf, Leipzig. Continuing through remaining 26 cities.</t>
         </is>
       </c>
     </row>
@@ -61102,7 +61102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J35"/>
+  <dimension ref="A1:J65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -62770,6 +62770,1416 @@
         </is>
       </c>
       <c r="I35" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Leipzig</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Lebensart Naturkost</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>http://www.lebensart-naturkost.de/</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Leipzig</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Naturkostladen Gohlis (Frickestraße 2)</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>https://www.naturkost-gohlis.de/</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Leipzig</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Bio-Flair</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>https://www.bio-flair.de/</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Leipzig</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Bio-Tempel</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>https://www.bio-tempel.de/</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Leipzig</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Bio-Mare (Plagwitz, Karl-Heine-Straße 43-45)</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>https://www.bio-mare.com/</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Leipzig</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Lindengrün Bioladen</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>https://www.lindengruen-bioladen.de/</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Leipzig</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Alnatura (Willy-Brandt-Platz 7)</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>https://www.alnatura.de/de-de/maerkte/marktseiten/leipzig/</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Leipzig</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Denns BioMarkt (Blochmannstr. 56)</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Leipzig</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Bio Company (Nikolaistraße 27-29, Zeppelinhaus)</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>https://www.biocompany.de/</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Leipzig</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Biomare (Connewitz, Simildenstr. 20)</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>https://www.bio-mare.com/</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Leipzig</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Biomare (Südvorstadt, Karl-Liebknecht-Str. 27)</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>https://www.bio-mare.com/</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Leipzig</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Schwarzwurzel OHG (Altlindenau)</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Leipzig</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Denns BioMarkt (Täubchenweg 22, Reudnitz)</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>https://www.biomarkt.de/leipzig-taeubchenweg-22-breitkopfstr/marktseite/</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Leipzig</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Unverpacktladen (Josephinenstraße 12, Reudnitz)</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Leipzig</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Denns BioMarkt (Höfe am Brühl)</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Leipzig</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Denns BioMarkt (Handelsstraße)</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Leipzig</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Denns BioMarkt (Karl-Liebknecht-Str. 8-14)</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>https://www.biomarkt.de/leipzig-karl-liebknecht-str-8-14/marktseite/</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Leipzig</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>BioKaufmannsladen (Gohliser Str. 40)</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>https://bio-kaufmannsladen.de/</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Leipzig</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Bioladen (Eisenbahnstraße 27, Neustadt-Neuschönefeld)</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Leipzig</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Kostbar Naturkost (Plagwitz)</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Leipzig</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Inge Blankenbach Vegetarische Spezialitäten (Böhlitz-Ehrenberg)</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>https://www.delikat-essen-in-leipzig.de/</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Leipzig</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Einfach Unverpackt</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>https://www.einfach-unverpackt.de/</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Leipzig</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Lieber lose (Plagwitz)</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Leipzig</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Bioladen (Hans-Poeche-Str. 2-4, Zentrum-Ost)</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Leipzig</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>natur &amp; fein (Waldstraße 23)</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Leipzig</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Biokarawane (Rossplatz)</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Leipzig</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Naturkostkontor Schreiter &amp; Co (Karl-Liebknecht-Str. 30-32)</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Leipzig</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Macis Markt (Markgrafenstr. 10)</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>https://macis-leipzig.de/</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Leipzig</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Locker lose</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Leipzig</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Bioladen (Städtelner Straße 62, Gohlis)</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>

</xml_diff>

<commit_message>
Add Bioladen data for Dortmund (>=30, name+website)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014Rwn272zpXB7zKQQT9xQTB
</commit_message>
<xml_diff>
--- a/outreach/ginger_shoc_outreach_tracker.xlsx
+++ b/outreach/ginger_shoc_outreach_tracker.xlsx
@@ -530,7 +530,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Bioladen expansion (2026-08-23): &gt;=30 per city, names+websites only. 7 of 33 done: Berlin, Hamburg, Munich, Cologne, Stuttgart, Düsseldorf, Leipzig. Continuing through remaining 26 cities.</t>
+          <t>Bioladen expansion (2026-08-23): &gt;=30 per city, names+websites only. 8 of 33 done: Berlin, Hamburg, Munich, Cologne, Stuttgart, Düsseldorf, Leipzig, Dortmund. Continuing through remaining 25 cities.</t>
         </is>
       </c>
     </row>
@@ -64196,7 +64196,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J34"/>
+  <dimension ref="A1:J64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -65817,6 +65817,1416 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Dortmund</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Kornhaus Naturkost (Lindemannstr. 14)</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>https://www.kornhaus-naturkost.de/</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Dortmund</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Aurum Bioladen (Aplerbeck)</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>https://www.aurum-bioladen.de/</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Dortmund</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>BasicBio (Kampstraße 102)</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>https://www.basicbio.de/</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Dortmund</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Fruchtbare Erde (Saarlandstr. 112)</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>https://www.fruchtbare-erde.de/</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Dortmund</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Fruchtbare Erde (Stockumer Str. 412)</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>https://www.fruchtbare-erde.de/</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Dortmund</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>AWO Schultenhof (Stockumer Str. 109)</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>https://www.awo-schultenhof.de/</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Dortmund</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Denns BioMarkt (Lindemannstr. 6-8)</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>https://www.biomarkt.de/dortmund-lindemannstr-6-8/marktseite/</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Dortmund</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Denns BioMarkt (Kaiserstr. 93)</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>https://www.biomarkt.de/dortmund-kaiserstr-93/marktseite/</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Dortmund</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>SuperBioMarkt (Brackel)</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>https://www.superbiomarkt.de/dortmund-brackel/</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Dortmund</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>SuperBioMarkt (Hombruch, Harkortstraße 18)</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>https://www.superbiomarkt.de/</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Dortmund</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>SuperBioMarkt (Hörde, Westfalendamm 285)</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>https://www.superbiomarkt.de/</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Dortmund</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Bioladen (Mergelteichstraße 47, Hombruch)</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Dortmund</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Grünkäppchen Natürlich Bio (Wickede)</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Dortmund</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Bioladen (Totilastr. 7, Huckarde)</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Dortmund</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Bioladen (Preinstraße 94, Wellinghofen)</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Dortmund</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Bioladen Sonnen-Naturkost Lunemann</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Dortmund</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Bövings Marktladen</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Dortmund</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Kornblume Naturkost</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Dortmund</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Bioladen Löwenzahn</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Dortmund</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Bioladen Kraftvoll</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Dortmund</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Bio-Garten (Dortmund)</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Dortmund</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Fruchtbare Erde (Eichlinghofen)</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>https://www.fruchtbare-erde.de/eichlinghofen.htm</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Dortmund</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Pur Bio (Saarlandstraße 118)</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>https://pur-bio.de/</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Dortmund</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Bioladen (Provinzialstr. 25-27, Lütgendortmund)</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Dortmund</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Naturkost Der Laden (Dortmund-Hörde)</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Dortmund</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Werkhof-Demeter-Gärtnerei mit Hofladen (Grevel)</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Dortmund</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Mein Biolädchen (Hagener Straße 341, Kirchhörde)</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Dortmund</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Bioladen (Wulfshofstr. 16, Oespel)</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Dortmund</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Fruchtbare Erde (Innenstadt-Süd)</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>https://www.fruchtbare-erde.de/innenstadt.htm</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Dortmund</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Bioladen</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>SuperBioMarkt (Gartenstadt)</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>https://www.superbiomarkt.de/dortmund-hoerde/</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>